<commit_message>
rerun model qwen3:8b RAG TOT Model results generated
</commit_message>
<xml_diff>
--- a/results/qwen3_8b/comparison_ToTRAG/ToTRAG_consolidated.xlsx
+++ b/results/qwen3_8b/comparison_ToTRAG/ToTRAG_consolidated.xlsx
@@ -545,46 +545,46 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.2037735809480954</v>
+        <v>0.2802850306640112</v>
       </c>
       <c r="D2" t="n">
-        <v>1.730519463176098e-79</v>
+        <v>0.04389910330770813</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5726922154426575</v>
+        <v>0.6463813781738281</v>
       </c>
       <c r="F2" t="n">
-        <v>27.79104591836736</v>
+        <v>49.51201581027669</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4304635761589404</v>
+        <v>1.364238410596027</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2513089005235602</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1836734693877551</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="N2" t="n">
-        <v>211.3978805541992</v>
+        <v>310.8729336261749</v>
       </c>
       <c r="O2" t="n">
-        <v>1423.0078125</v>
+        <v>1440.953125</v>
       </c>
       <c r="P2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Q2" t="n">
         <v>20</v>
@@ -593,10 +593,10 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>0.9461557865142822</v>
+        <v>1.202955007553101</v>
       </c>
       <c r="T2" t="n">
-        <v>210.4517211914062</v>
+        <v>309.6699740886688</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -612,46 +612,46 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.09708737688754834</v>
+        <v>0.114754096855684</v>
       </c>
       <c r="D3" t="n">
-        <v>1.902237782330245e-155</v>
+        <v>8.709768942723901e-232</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4620912075042725</v>
+        <v>0.4636981785297394</v>
       </c>
       <c r="F3" t="n">
-        <v>28.62210798122067</v>
+        <v>9.884166666666715</v>
       </c>
       <c r="G3" t="n">
-        <v>5.073394495412844</v>
+        <v>5.954128440366972</v>
       </c>
       <c r="H3" t="n">
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.2043010752688172</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2647058823529412</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="N3" t="n">
-        <v>178.1337730884552</v>
+        <v>167.1431570053101</v>
       </c>
       <c r="O3" t="n">
-        <v>1423.21484375</v>
+        <v>1441.18359375</v>
       </c>
       <c r="P3" t="n">
-        <v>13.2</v>
+        <v>13.7</v>
       </c>
       <c r="Q3" t="n">
         <v>20</v>
@@ -660,10 +660,10 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>1.448410034179688</v>
+        <v>1.503925800323486</v>
       </c>
       <c r="T3" t="n">
-        <v>176.6853597164154</v>
+        <v>165.639228105545</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -679,19 +679,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.2460317413151928</v>
+        <v>0.2996254633068216</v>
       </c>
       <c r="D4" t="n">
-        <v>5.219478241687084e-79</v>
+        <v>0.01901847649876204</v>
       </c>
       <c r="E4" t="n">
-        <v>0.5399104952812195</v>
+        <v>0.5807259082794189</v>
       </c>
       <c r="F4" t="n">
-        <v>37.91352906050957</v>
+        <v>55.81330039525693</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6217948717948718</v>
+        <v>0.6805555555555556</v>
       </c>
       <c r="H4" t="n">
         <v>0.5</v>
@@ -703,22 +703,22 @@
         <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.2926829268292683</v>
+        <v>0.3225806451612903</v>
       </c>
       <c r="M4" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.3243243243243243</v>
       </c>
       <c r="N4" t="n">
-        <v>148.4784555435181</v>
+        <v>202.0801162719727</v>
       </c>
       <c r="O4" t="n">
-        <v>1423.21875</v>
+        <v>1441.3828125</v>
       </c>
       <c r="P4" t="n">
-        <v>13.2</v>
+        <v>13.5</v>
       </c>
       <c r="Q4" t="n">
         <v>20</v>
@@ -727,10 +727,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>1.32028603553772</v>
+        <v>1.309788465499878</v>
       </c>
       <c r="T4" t="n">
-        <v>147.1581671237946</v>
+        <v>200.770325422287</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -746,22 +746,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.156996583188622</v>
+        <v>0.1783439447748388</v>
       </c>
       <c r="D5" t="n">
-        <v>2.098152133550718e-156</v>
+        <v>0.005446929611769897</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6534578204154968</v>
+        <v>0.5241946578025818</v>
       </c>
       <c r="F5" t="n">
-        <v>36.4156730769231</v>
+        <v>25.23000000000005</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4108019639934534</v>
+        <v>0.486088379705401</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
@@ -770,22 +770,22 @@
         <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>0.2950819672131147</v>
+        <v>0.3012048192771085</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2391304347826087</v>
+        <v>0.1566265060240964</v>
       </c>
       <c r="N5" t="n">
-        <v>183.1602656841278</v>
+        <v>189.0723538398743</v>
       </c>
       <c r="O5" t="n">
-        <v>1423.37109375</v>
+        <v>1442.5859375</v>
       </c>
       <c r="P5" t="n">
-        <v>13.3</v>
+        <v>13.5</v>
       </c>
       <c r="Q5" t="n">
         <v>20</v>
@@ -794,10 +794,10 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>1.461454153060913</v>
+        <v>1.206163644790649</v>
       </c>
       <c r="T5" t="n">
-        <v>181.698807477951</v>
+        <v>187.866188287735</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -813,22 +813,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.3247863202337644</v>
+        <v>0.2407407365706448</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01992435169682143</v>
+        <v>2.282216633601617e-79</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6595125794410706</v>
+        <v>0.5687358379364014</v>
       </c>
       <c r="F6" t="n">
-        <v>53.39331250000001</v>
+        <v>37.45538461538465</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5678160919540229</v>
+        <v>0.4597701149425287</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
@@ -840,19 +840,19 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>0.2424242424242424</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2647058823529412</v>
+        <v>0.1397849462365592</v>
       </c>
       <c r="N6" t="n">
-        <v>143.5443737506866</v>
+        <v>161.7180795669556</v>
       </c>
       <c r="O6" t="n">
-        <v>1423.515625</v>
+        <v>1442.84765625</v>
       </c>
       <c r="P6" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="Q6" t="n">
         <v>20</v>
@@ -861,10 +861,10 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>1.243539571762085</v>
+        <v>1.223984956741333</v>
       </c>
       <c r="T6" t="n">
-        <v>142.3008322715759</v>
+        <v>160.4940919876099</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -880,46 +880,46 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.2247190977838811</v>
+        <v>0.1614906796071236</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0009973721376269843</v>
+        <v>0.0002373577558022702</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6286501288414001</v>
+        <v>0.6024760603904724</v>
       </c>
       <c r="F7" t="n">
-        <v>-52.6211764705882</v>
+        <v>-6.796126027397264</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2522548734361362</v>
+        <v>0.2900785568810009</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>0.1764705882352941</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
         <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1652173913043478</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="M7" t="n">
-        <v>0.53125</v>
+        <v>0.4845360824742268</v>
       </c>
       <c r="N7" t="n">
-        <v>331.4431223869324</v>
+        <v>305.1571083068848</v>
       </c>
       <c r="O7" t="n">
-        <v>1424.984375</v>
+        <v>1443.47265625</v>
       </c>
       <c r="P7" t="n">
-        <v>13.4</v>
+        <v>13.9</v>
       </c>
       <c r="Q7" t="n">
         <v>20</v>
@@ -928,10 +928,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>1.218279600143433</v>
+        <v>1.205789089202881</v>
       </c>
       <c r="T7" t="n">
-        <v>330.2248401641846</v>
+        <v>303.9513173103333</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -947,46 +947,46 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.07604562506903388</v>
+        <v>0.2043343611728284</v>
       </c>
       <c r="D8" t="n">
-        <v>8.122503374890562e-161</v>
+        <v>0.003580694026239782</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5455583930015564</v>
+        <v>0.6190401315689087</v>
       </c>
       <c r="F8" t="n">
-        <v>-2.315467479674766</v>
+        <v>25.44431721798136</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1965277777777778</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2</v>
+        <v>0.35</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" t="n">
         <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="L8" t="n">
-        <v>0.3928571428571428</v>
+        <v>0.3292682926829268</v>
       </c>
       <c r="M8" t="n">
-        <v>0.07894736842105263</v>
+        <v>0.1176470588235294</v>
       </c>
       <c r="N8" t="n">
-        <v>285.5549674034119</v>
+        <v>177.4175817966461</v>
       </c>
       <c r="O8" t="n">
-        <v>1424.984375</v>
+        <v>1443.6015625</v>
       </c>
       <c r="P8" t="n">
-        <v>13.4</v>
+        <v>13.5</v>
       </c>
       <c r="Q8" t="n">
         <v>20</v>
@@ -995,10 +995,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>1.554473638534546</v>
+        <v>1.230495691299438</v>
       </c>
       <c r="T8" t="n">
-        <v>284.0004913806915</v>
+        <v>176.1870834827423</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -1014,19 +1014,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.1581920871216765</v>
+        <v>0.1758241723036168</v>
       </c>
       <c r="D9" t="n">
-        <v>3.89003801738445e-157</v>
+        <v>8.008054613384905e-157</v>
       </c>
       <c r="E9" t="n">
-        <v>0.5182662010192871</v>
+        <v>0.5668753981590271</v>
       </c>
       <c r="F9" t="n">
-        <v>50.70362211221124</v>
+        <v>40.48591176470592</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2236384704519119</v>
+        <v>0.2734646581691773</v>
       </c>
       <c r="H9" t="n">
         <v>0.125</v>
@@ -1041,19 +1041,19 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>0.3225806451612903</v>
+        <v>0.3287671232876712</v>
       </c>
       <c r="M9" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.1358024691358025</v>
       </c>
       <c r="N9" t="n">
-        <v>209.1037220954895</v>
+        <v>201.1769127845764</v>
       </c>
       <c r="O9" t="n">
-        <v>1424.984375</v>
+        <v>1443.60546875</v>
       </c>
       <c r="P9" t="n">
-        <v>13.3</v>
+        <v>13.5</v>
       </c>
       <c r="Q9" t="n">
         <v>20</v>
@@ -1062,10 +1062,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>1.291558504104614</v>
+        <v>1.249756097793579</v>
       </c>
       <c r="T9" t="n">
-        <v>207.8121614456177</v>
+        <v>199.9271540641785</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -1081,19 +1081,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.1056338001500199</v>
+        <v>0.1628664460626638</v>
       </c>
       <c r="D10" t="n">
-        <v>1.394605555319197e-158</v>
+        <v>2.140753119986657e-80</v>
       </c>
       <c r="E10" t="n">
-        <v>0.5722618699073792</v>
+        <v>0.582069456577301</v>
       </c>
       <c r="F10" t="n">
-        <v>29.26333333333335</v>
+        <v>43.62325091575093</v>
       </c>
       <c r="G10" t="n">
-        <v>0.212962962962963</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="H10" t="n">
         <v>0.3125</v>
@@ -1102,25 +1102,25 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>0.325</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2079207920792079</v>
+        <v>0.09722222222222221</v>
       </c>
       <c r="N10" t="n">
-        <v>196.254499912262</v>
+        <v>195.3745613098145</v>
       </c>
       <c r="O10" t="n">
-        <v>1424.984375</v>
+        <v>1443.6875</v>
       </c>
       <c r="P10" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="Q10" t="n">
         <v>20</v>
@@ -1129,10 +1129,10 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>1.228546142578125</v>
+        <v>1.255224704742432</v>
       </c>
       <c r="T10" t="n">
-        <v>195.0259521007538</v>
+        <v>194.1193339824677</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1148,22 +1148,22 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.1564245779630786</v>
+        <v>0.1889763743443487</v>
       </c>
       <c r="D11" t="n">
-        <v>7.551042687299704e-158</v>
+        <v>6.432609166628714e-157</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5625163912773132</v>
+        <v>0.5794017314910889</v>
       </c>
       <c r="F11" t="n">
-        <v>40.02130645161293</v>
+        <v>35.70607142857145</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2203389830508475</v>
+        <v>0.2837616183706944</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2777777777777778</v>
       </c>
       <c r="I11" t="n">
         <v>1</v>
@@ -1175,19 +1175,19 @@
         <v>0.5</v>
       </c>
       <c r="L11" t="n">
-        <v>0.3928571428571428</v>
+        <v>0.358974358974359</v>
       </c>
       <c r="M11" t="n">
-        <v>0.1588785046728972</v>
+        <v>0.1836734693877551</v>
       </c>
       <c r="N11" t="n">
-        <v>202.4620254039764</v>
+        <v>207.230345249176</v>
       </c>
       <c r="O11" t="n">
-        <v>1424.984375</v>
+        <v>1443.6953125</v>
       </c>
       <c r="P11" t="n">
-        <v>13.1</v>
+        <v>13.7</v>
       </c>
       <c r="Q11" t="n">
         <v>20</v>
@@ -1196,10 +1196,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>1.489540576934814</v>
+        <v>1.271144151687622</v>
       </c>
       <c r="T11" t="n">
-        <v>200.972482919693</v>
+        <v>205.9591982364655</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1215,19 +1215,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.2210796875056338</v>
+        <v>0.2739725981404684</v>
       </c>
       <c r="D12" t="n">
-        <v>0.004668335673030102</v>
+        <v>0.06200097980716292</v>
       </c>
       <c r="E12" t="n">
-        <v>0.65522301197052</v>
+        <v>0.6635017991065979</v>
       </c>
       <c r="F12" t="n">
-        <v>35.73416666666668</v>
+        <v>46.73448717948722</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3758542141230068</v>
+        <v>0.6007972665148064</v>
       </c>
       <c r="H12" t="n">
         <v>0.3333333333333333</v>
@@ -1236,25 +1236,25 @@
         <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L12" t="n">
-        <v>0.247191011235955</v>
+        <v>0.2945736434108527</v>
       </c>
       <c r="M12" t="n">
-        <v>0.1608391608391608</v>
+        <v>0.375</v>
       </c>
       <c r="N12" t="n">
-        <v>204.6425461769104</v>
+        <v>235.5697114467621</v>
       </c>
       <c r="O12" t="n">
-        <v>1424.984375</v>
+        <v>1443.7578125</v>
       </c>
       <c r="P12" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="Q12" t="n">
         <v>20</v>
@@ -1263,10 +1263,10 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>1.255172967910767</v>
+        <v>1.214060306549072</v>
       </c>
       <c r="T12" t="n">
-        <v>203.3873710632324</v>
+        <v>234.3556480407715</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -1282,22 +1282,22 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.1288515377827995</v>
+        <v>0.1658031052323553</v>
       </c>
       <c r="D13" t="n">
-        <v>5.119788514303341e-158</v>
+        <v>7.10711879349888e-81</v>
       </c>
       <c r="E13" t="n">
-        <v>0.5463192462921143</v>
+        <v>0.6234800219535828</v>
       </c>
       <c r="F13" t="n">
-        <v>38.38505494505497</v>
+        <v>31.70302631578949</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2039911308203991</v>
+        <v>0.2954545454545455</v>
       </c>
       <c r="H13" t="n">
-        <v>0.15</v>
+        <v>0.45</v>
       </c>
       <c r="I13" t="n">
         <v>1</v>
@@ -1309,19 +1309,19 @@
         <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>0.2777777777777778</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1463414634146341</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="N13" t="n">
-        <v>183.3079771995544</v>
+        <v>199.3811047077179</v>
       </c>
       <c r="O13" t="n">
-        <v>1424.984375</v>
+        <v>1443.7578125</v>
       </c>
       <c r="P13" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="Q13" t="n">
         <v>20</v>
@@ -1330,10 +1330,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>1.484333276748657</v>
+        <v>1.250001907348633</v>
       </c>
       <c r="T13" t="n">
-        <v>181.8236410617828</v>
+        <v>198.1311006546021</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1349,19 +1349,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.1730279859539396</v>
+        <v>0.1303116117985058</v>
       </c>
       <c r="D14" t="n">
-        <v>0.002124415352444144</v>
+        <v>5.763632549867579e-158</v>
       </c>
       <c r="E14" t="n">
-        <v>0.5984796285629272</v>
+        <v>0.5841918587684631</v>
       </c>
       <c r="F14" t="n">
-        <v>40.87176804286167</v>
+        <v>27.69384615384618</v>
       </c>
       <c r="G14" t="n">
-        <v>0.365</v>
+        <v>0.2433333333333333</v>
       </c>
       <c r="H14" t="n">
         <v>0.3</v>
@@ -1370,25 +1370,25 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.3272727272727273</v>
       </c>
       <c r="M14" t="n">
-        <v>0.2086330935251799</v>
+        <v>0.2125984251968504</v>
       </c>
       <c r="N14" t="n">
-        <v>238.224672794342</v>
+        <v>165.5595126152039</v>
       </c>
       <c r="O14" t="n">
-        <v>1424.984375</v>
+        <v>1443.7578125</v>
       </c>
       <c r="P14" t="n">
-        <v>13</v>
+        <v>13.3</v>
       </c>
       <c r="Q14" t="n">
         <v>20</v>
@@ -1397,10 +1397,10 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>1.296699523925781</v>
+        <v>1.259896755218506</v>
       </c>
       <c r="T14" t="n">
-        <v>236.9279713630676</v>
+        <v>164.2996129989624</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -1416,19 +1416,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.2694300468200489</v>
+        <v>0.2716049335467155</v>
       </c>
       <c r="D15" t="n">
-        <v>0.04233597443220442</v>
+        <v>0.06168908678404924</v>
       </c>
       <c r="E15" t="n">
-        <v>0.6549957394599915</v>
+        <v>0.6621700525283813</v>
       </c>
       <c r="F15" t="n">
-        <v>66.35845368916799</v>
+        <v>66.5904166666667</v>
       </c>
       <c r="G15" t="n">
-        <v>1.13682092555332</v>
+        <v>0.7947686116700201</v>
       </c>
       <c r="H15" t="n">
         <v>0.5</v>
@@ -1440,22 +1440,22 @@
         <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L15" t="n">
-        <v>0.46875</v>
+        <v>0.3</v>
       </c>
       <c r="M15" t="n">
-        <v>0.2452830188679246</v>
+        <v>0.1596638655462185</v>
       </c>
       <c r="N15" t="n">
-        <v>202.8805346488953</v>
+        <v>146.7446558475494</v>
       </c>
       <c r="O15" t="n">
-        <v>1424.984375</v>
+        <v>1443.76171875</v>
       </c>
       <c r="P15" t="n">
-        <v>13.4</v>
+        <v>13.7</v>
       </c>
       <c r="Q15" t="n">
         <v>20</v>
@@ -1464,10 +1464,10 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>1.465949296951294</v>
+        <v>1.292887210845947</v>
       </c>
       <c r="T15" t="n">
-        <v>201.4145829677582</v>
+        <v>145.4517657756805</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -1483,19 +1483,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.334728028504403</v>
+        <v>0.2953586448282862</v>
       </c>
       <c r="D16" t="n">
-        <v>0.02719889876789828</v>
+        <v>4.143346747104959e-155</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6745786070823669</v>
+        <v>0.6433549523353577</v>
       </c>
       <c r="F16" t="n">
-        <v>54.39610759493675</v>
+        <v>51.55000000000004</v>
       </c>
       <c r="G16" t="n">
-        <v>0.8972895863052782</v>
+        <v>0.8801711840228246</v>
       </c>
       <c r="H16" t="n">
         <v>0.4</v>
@@ -1507,22 +1507,22 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0.2771084337349398</v>
+        <v>0.3950617283950617</v>
       </c>
       <c r="M16" t="n">
-        <v>0.3043478260869565</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="N16" t="n">
-        <v>184.6559479236603</v>
+        <v>155.9911365509033</v>
       </c>
       <c r="O16" t="n">
-        <v>1424.984375</v>
+        <v>1443.765625</v>
       </c>
       <c r="P16" t="n">
-        <v>13.3</v>
+        <v>13.6</v>
       </c>
       <c r="Q16" t="n">
         <v>20</v>
@@ -1531,10 +1531,10 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>1.216969966888428</v>
+        <v>1.258129835128784</v>
       </c>
       <c r="T16" t="n">
-        <v>183.4389758110046</v>
+        <v>154.7330040931702</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -1550,19 +1550,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.2417582367588457</v>
+        <v>0.307692302735662</v>
       </c>
       <c r="D17" t="n">
-        <v>6.923169578399921e-79</v>
+        <v>4.483793999855553e-155</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6635465621948242</v>
+        <v>0.6779084801673889</v>
       </c>
       <c r="F17" t="n">
-        <v>65.86748931623936</v>
+        <v>50.62711233885818</v>
       </c>
       <c r="G17" t="n">
-        <v>1.19758064516129</v>
+        <v>0.8830645161290323</v>
       </c>
       <c r="H17" t="n">
         <v>0.2857142857142857</v>
@@ -1571,22 +1571,22 @@
         <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" t="n">
-        <v>0.2755102040816326</v>
+        <v>0.3132530120481928</v>
       </c>
       <c r="M17" t="n">
-        <v>0.3449781659388647</v>
+        <v>0.25</v>
       </c>
       <c r="N17" t="n">
-        <v>225.6616806983948</v>
+        <v>176.6943078041077</v>
       </c>
       <c r="O17" t="n">
-        <v>1424.98828125</v>
+        <v>1443.82421875</v>
       </c>
       <c r="P17" t="n">
         <v>13.5</v>
@@ -1598,10 +1598,10 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>1.252410888671875</v>
+        <v>1.258592844009399</v>
       </c>
       <c r="T17" t="n">
-        <v>224.4092671871185</v>
+        <v>175.4357128143311</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
@@ -1617,22 +1617,22 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.1545064352453536</v>
+        <v>0.198412695068106</v>
       </c>
       <c r="D18" t="n">
-        <v>7.329163753806349e-05</v>
+        <v>0.001537731997565385</v>
       </c>
       <c r="E18" t="n">
-        <v>0.5975859761238098</v>
+        <v>0.6199045181274414</v>
       </c>
       <c r="F18" t="n">
-        <v>42.52500000000001</v>
+        <v>50.2376315789474</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1647196261682243</v>
+        <v>0.2605140186915888</v>
       </c>
       <c r="H18" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I18" t="n">
         <v>1</v>
@@ -1644,19 +1644,19 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0.1754385964912281</v>
+        <v>0.2934782608695652</v>
       </c>
       <c r="M18" t="n">
-        <v>0.1752577319587629</v>
+        <v>0.2452830188679246</v>
       </c>
       <c r="N18" t="n">
-        <v>181.3436617851257</v>
+        <v>236.8438758850098</v>
       </c>
       <c r="O18" t="n">
-        <v>1424.98828125</v>
+        <v>1443.828125</v>
       </c>
       <c r="P18" t="n">
-        <v>13.4</v>
+        <v>13.9</v>
       </c>
       <c r="Q18" t="n">
         <v>20</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>1.27207088470459</v>
+        <v>1.245406150817871</v>
       </c>
       <c r="T18" t="n">
-        <v>180.0715887546539</v>
+        <v>235.5984673500061</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
@@ -1684,22 +1684,22 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.121387279103044</v>
+        <v>0.1437908464810544</v>
       </c>
       <c r="D19" t="n">
-        <v>2.862751418642962e-156</v>
+        <v>8.508076552407284e-82</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6129412055015564</v>
+        <v>0.5815699100494385</v>
       </c>
       <c r="F19" t="n">
-        <v>4.490693363520592</v>
+        <v>16.95392156862749</v>
       </c>
       <c r="G19" t="n">
-        <v>0.4792353328938695</v>
+        <v>0.2682926829268293</v>
       </c>
       <c r="H19" t="n">
-        <v>0.6470588235294118</v>
+        <v>0.2352941176470588</v>
       </c>
       <c r="I19" t="n">
         <v>1</v>
@@ -1711,19 +1711,19 @@
         <v>0.5</v>
       </c>
       <c r="L19" t="n">
-        <v>0.25</v>
+        <v>0.2407407407407407</v>
       </c>
       <c r="M19" t="n">
-        <v>0.2244897959183673</v>
+        <v>0.09677419354838709</v>
       </c>
       <c r="N19" t="n">
-        <v>252.1928403377533</v>
+        <v>182.3371558189392</v>
       </c>
       <c r="O19" t="n">
-        <v>1424.98828125</v>
+        <v>1443.83203125</v>
       </c>
       <c r="P19" t="n">
-        <v>13.4</v>
+        <v>13.6</v>
       </c>
       <c r="Q19" t="n">
         <v>20</v>
@@ -1732,10 +1732,10 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>1.243606805801392</v>
+        <v>1.275394916534424</v>
       </c>
       <c r="T19" t="n">
-        <v>250.949230670929</v>
+        <v>181.061758518219</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -1751,46 +1751,46 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.1924398598344375</v>
+        <v>0.2291021634874293</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0002754883808062679</v>
+        <v>0.004646776935916677</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6416764259338379</v>
+        <v>0.5817007422447205</v>
       </c>
       <c r="F20" t="n">
-        <v>51.70795698924732</v>
+        <v>49.96476190476193</v>
       </c>
       <c r="G20" t="n">
-        <v>0.220014194464159</v>
+        <v>0.3151171043293116</v>
       </c>
       <c r="H20" t="n">
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
         <v>0.5</v>
       </c>
       <c r="L20" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.3134328358208955</v>
       </c>
       <c r="M20" t="n">
-        <v>0.1129032258064516</v>
+        <v>0.126984126984127</v>
       </c>
       <c r="N20" t="n">
-        <v>195.9814608097076</v>
+        <v>187.0562489032745</v>
       </c>
       <c r="O20" t="n">
-        <v>1424.98828125</v>
+        <v>1443.83203125</v>
       </c>
       <c r="P20" t="n">
-        <v>13.5</v>
+        <v>13.4</v>
       </c>
       <c r="Q20" t="n">
         <v>20</v>
@@ -1799,10 +1799,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>1.453266859054565</v>
+        <v>1.238818168640137</v>
       </c>
       <c r="T20" t="n">
-        <v>194.5281913280487</v>
+        <v>185.8174278736115</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -1818,19 +1818,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.1111111084659747</v>
+        <v>0.102893887847727</v>
       </c>
       <c r="D21" t="n">
-        <v>5.193780808598403e-83</v>
+        <v>2.312405001485916e-158</v>
       </c>
       <c r="E21" t="n">
-        <v>0.5604392886161804</v>
+        <v>0.4981350302696228</v>
       </c>
       <c r="F21" t="n">
-        <v>28.23966666666669</v>
+        <v>30.47756147540989</v>
       </c>
       <c r="G21" t="n">
-        <v>0.175070821529745</v>
+        <v>0.1807365439093484</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1839,25 +1839,25 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.125</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.3023255813953488</v>
       </c>
       <c r="M21" t="n">
-        <v>0.0339425587467363</v>
+        <v>0.05511811023622047</v>
       </c>
       <c r="N21" t="n">
-        <v>184.6234850883484</v>
+        <v>275.7304401397705</v>
       </c>
       <c r="O21" t="n">
-        <v>1424.98828125</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P21" t="n">
-        <v>13.2</v>
+        <v>13.5</v>
       </c>
       <c r="Q21" t="n">
         <v>20</v>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>1.478805065155029</v>
+        <v>1.421154975891113</v>
       </c>
       <c r="T21" t="n">
-        <v>183.144677400589</v>
+        <v>274.3092832565308</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -1885,46 +1885,46 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.3436754128969418</v>
+        <v>0.3359374950000763</v>
       </c>
       <c r="D22" t="n">
-        <v>0.05294600622677436</v>
+        <v>0.07053867871481319</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6309255957603455</v>
+        <v>0.6660435795783997</v>
       </c>
       <c r="F22" t="n">
-        <v>43.69674661866304</v>
+        <v>47.30143659711078</v>
       </c>
       <c r="G22" t="n">
-        <v>0.703030303030303</v>
+        <v>1.118181818181818</v>
       </c>
       <c r="H22" t="n">
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
       <c r="I22" t="n">
         <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>0.2605633802816901</v>
+        <v>0.2712765957446808</v>
       </c>
       <c r="M22" t="n">
-        <v>0.4186046511627907</v>
+        <v>0.5633187772925764</v>
       </c>
       <c r="N22" t="n">
-        <v>171.9529812335968</v>
+        <v>196.696005821228</v>
       </c>
       <c r="O22" t="n">
-        <v>1424.98828125</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P22" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="Q22" t="n">
         <v>20</v>
@@ -1933,10 +1933,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>1.472054004669189</v>
+        <v>1.471139430999756</v>
       </c>
       <c r="T22" t="n">
-        <v>170.4809243679047</v>
+        <v>195.2248642444611</v>
       </c>
       <c r="U22" t="n">
         <v>0</v>
@@ -1952,46 +1952,46 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.3326885834688297</v>
+        <v>0.279441113360664</v>
       </c>
       <c r="D23" t="n">
-        <v>0.04283608159216823</v>
+        <v>0.006602789951994124</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6378268599510193</v>
+        <v>0.6492375135421753</v>
       </c>
       <c r="F23" t="n">
-        <v>35.1320666666667</v>
+        <v>21.45194612794617</v>
       </c>
       <c r="G23" t="n">
-        <v>0.5548920532843362</v>
+        <v>0.4598070739549839</v>
       </c>
       <c r="H23" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>0.5</v>
+        <v>0.85</v>
       </c>
       <c r="L23" t="n">
-        <v>0.2214765100671141</v>
+        <v>0.2357142857142857</v>
       </c>
       <c r="M23" t="n">
-        <v>0.5804195804195804</v>
+        <v>0.3269230769230769</v>
       </c>
       <c r="N23" t="n">
-        <v>248.1762750148773</v>
+        <v>186.1756653785706</v>
       </c>
       <c r="O23" t="n">
-        <v>1424.98828125</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P23" t="n">
-        <v>13.3</v>
+        <v>13.6</v>
       </c>
       <c r="Q23" t="n">
         <v>20</v>
@@ -2000,10 +2000,10 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>1.248279809951782</v>
+        <v>1.253982782363892</v>
       </c>
       <c r="T23" t="n">
-        <v>246.9279928207397</v>
+        <v>184.9216799736023</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.314049581875555</v>
+        <v>0.2488038227513107</v>
       </c>
       <c r="D24" t="n">
-        <v>4.317821519005071e-155</v>
+        <v>1.109142043699342e-78</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6371414065361023</v>
+        <v>0.6110427975654602</v>
       </c>
       <c r="F24" t="n">
-        <v>42.95136039250673</v>
+        <v>41.06107843137258</v>
       </c>
       <c r="G24" t="n">
-        <v>1.225806451612903</v>
+        <v>1.004608294930876</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
         <v>1</v>
@@ -2043,22 +2043,22 @@
         <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>0.3119266055045872</v>
+        <v>0.2777777777777778</v>
       </c>
       <c r="M24" t="n">
-        <v>0.3693693693693694</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="N24" t="n">
-        <v>153.3569903373718</v>
+        <v>139.8938827514648</v>
       </c>
       <c r="O24" t="n">
-        <v>1424.98828125</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P24" t="n">
-        <v>13.3</v>
+        <v>13.5</v>
       </c>
       <c r="Q24" t="n">
         <v>20</v>
@@ -2067,10 +2067,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>1.231390714645386</v>
+        <v>1.265970945358276</v>
       </c>
       <c r="T24" t="n">
-        <v>152.1255972385406</v>
+        <v>138.627908706665</v>
       </c>
       <c r="U24" t="n">
         <v>0</v>
@@ -2086,22 +2086,22 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.2527472480394881</v>
+        <v>0.3410138198933934</v>
       </c>
       <c r="D25" t="n">
-        <v>6.182703348071608e-79</v>
+        <v>0.03496693890036816</v>
       </c>
       <c r="E25" t="n">
-        <v>0.6571572422981262</v>
+        <v>0.6924597024917603</v>
       </c>
       <c r="F25" t="n">
-        <v>26.96450653120468</v>
+        <v>42.0577097902098</v>
       </c>
       <c r="G25" t="n">
-        <v>0.6817496229260935</v>
+        <v>0.9079939668174962</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
         <v>1</v>
@@ -2113,19 +2113,19 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>0.2280701754385965</v>
+        <v>0.3048780487804878</v>
       </c>
       <c r="M25" t="n">
-        <v>0.1791044776119403</v>
+        <v>0.358974358974359</v>
       </c>
       <c r="N25" t="n">
-        <v>195.9576551914215</v>
+        <v>201.1525661945343</v>
       </c>
       <c r="O25" t="n">
-        <v>1424.98828125</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P25" t="n">
-        <v>13.3</v>
+        <v>13.8</v>
       </c>
       <c r="Q25" t="n">
         <v>20</v>
@@ -2134,10 +2134,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>1.414610385894775</v>
+        <v>1.27272629737854</v>
       </c>
       <c r="T25" t="n">
-        <v>194.5430421829224</v>
+        <v>199.8798377513885</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2153,19 +2153,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.3648648602675311</v>
+        <v>0.2564102516477647</v>
       </c>
       <c r="D26" t="n">
-        <v>0.02483428507458189</v>
+        <v>5.254232059758959e-79</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6959307193756104</v>
+        <v>0.643599271774292</v>
       </c>
       <c r="F26" t="n">
-        <v>40.12</v>
+        <v>35.00192307692311</v>
       </c>
       <c r="G26" t="n">
-        <v>0.6273830155979203</v>
+        <v>0.6672443674176777</v>
       </c>
       <c r="H26" t="n">
         <v>1</v>
@@ -2180,19 +2180,19 @@
         <v>0.5</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2439024390243902</v>
+        <v>0.2884615384615384</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2424242424242424</v>
+        <v>0.2</v>
       </c>
       <c r="N26" t="n">
-        <v>162.7423067092896</v>
+        <v>161.6218037605286</v>
       </c>
       <c r="O26" t="n">
-        <v>1424.98828125</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P26" t="n">
-        <v>13.3</v>
+        <v>13.6</v>
       </c>
       <c r="Q26" t="n">
         <v>20</v>
@@ -2201,10 +2201,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>1.257335662841797</v>
+        <v>1.283930540084839</v>
       </c>
       <c r="T26" t="n">
-        <v>161.484968662262</v>
+        <v>160.3378708362579</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>
@@ -2220,46 +2220,46 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.278846149090699</v>
+        <v>0.3041474605831511</v>
       </c>
       <c r="D27" t="n">
-        <v>2.084154085234521e-155</v>
+        <v>1.002007873606135e-78</v>
       </c>
       <c r="E27" t="n">
-        <v>0.6353515982627869</v>
+        <v>0.6967757344245911</v>
       </c>
       <c r="F27" t="n">
-        <v>38.83097706032288</v>
+        <v>27.20235772357725</v>
       </c>
       <c r="G27" t="n">
-        <v>0.6716826265389877</v>
+        <v>0.6949384404924761</v>
       </c>
       <c r="H27" t="n">
         <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" t="n">
         <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L27" t="n">
-        <v>0.2463768115942029</v>
+        <v>0.3382352941176471</v>
       </c>
       <c r="M27" t="n">
-        <v>0.2134831460674157</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="N27" t="n">
-        <v>178.2678775787354</v>
+        <v>128.6752142906189</v>
       </c>
       <c r="O27" t="n">
-        <v>1424.98828125</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P27" t="n">
-        <v>13.2</v>
+        <v>13.5</v>
       </c>
       <c r="Q27" t="n">
         <v>20</v>
@@ -2268,10 +2268,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>1.450373649597168</v>
+        <v>1.421056509017944</v>
       </c>
       <c r="T27" t="n">
-        <v>176.817501783371</v>
+        <v>127.254154920578</v>
       </c>
       <c r="U27" t="n">
         <v>0</v>
@@ -2287,22 +2287,22 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.3246073250108276</v>
+        <v>0.3482142807146843</v>
       </c>
       <c r="D28" t="n">
-        <v>1.493969587489462e-78</v>
+        <v>0.06131338182016789</v>
       </c>
       <c r="E28" t="n">
-        <v>0.6791049838066101</v>
+        <v>0.7270402908325195</v>
       </c>
       <c r="F28" t="n">
-        <v>49.63168010752693</v>
+        <v>44.13137800687289</v>
       </c>
       <c r="G28" t="n">
-        <v>0.7727272727272727</v>
+        <v>1.053030303030303</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
         <v>1</v>
@@ -2314,19 +2314,19 @@
         <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>0.3103448275862069</v>
+        <v>0.2954545454545455</v>
       </c>
       <c r="M28" t="n">
-        <v>0.2708333333333334</v>
+        <v>0.3406593406593407</v>
       </c>
       <c r="N28" t="n">
-        <v>192.0386333465576</v>
+        <v>164.7901599407196</v>
       </c>
       <c r="O28" t="n">
-        <v>1424.9921875</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P28" t="n">
-        <v>13.4</v>
+        <v>13.7</v>
       </c>
       <c r="Q28" t="n">
         <v>20</v>
@@ -2335,10 +2335,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>1.255966186523438</v>
+        <v>1.232701539993286</v>
       </c>
       <c r="T28" t="n">
-        <v>190.782665014267</v>
+        <v>163.5574557781219</v>
       </c>
       <c r="U28" t="n">
         <v>0</v>
@@ -2354,22 +2354,22 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.2890173360887434</v>
+        <v>0.3290043241618411</v>
       </c>
       <c r="D29" t="n">
-        <v>1.373248971716225e-78</v>
+        <v>0.03606300935643239</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6453489065170288</v>
+        <v>0.705970823764801</v>
       </c>
       <c r="F29" t="n">
-        <v>53.77121621621623</v>
+        <v>52.49662105263161</v>
       </c>
       <c r="G29" t="n">
-        <v>0.875</v>
+        <v>1.418402777777778</v>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
         <v>1</v>
@@ -2378,19 +2378,19 @@
         <v>1</v>
       </c>
       <c r="K29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.2452830188679245</v>
       </c>
       <c r="M29" t="n">
-        <v>0.3023255813953489</v>
+        <v>0.3577981651376147</v>
       </c>
       <c r="N29" t="n">
-        <v>165.5448276996613</v>
+        <v>161.3088953495026</v>
       </c>
       <c r="O29" t="n">
-        <v>1424.9921875</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P29" t="n">
         <v>13.4</v>
@@ -2402,10 +2402,10 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>1.487584352493286</v>
+        <v>1.199329614639282</v>
       </c>
       <c r="T29" t="n">
-        <v>164.0572414398193</v>
+        <v>160.1095628738403</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
@@ -2421,46 +2421,46 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.09756097365556221</v>
+        <v>0.08108107993882398</v>
       </c>
       <c r="D30" t="n">
-        <v>2.073574161459504e-155</v>
+        <v>1.686106711860657e-155</v>
       </c>
       <c r="E30" t="n">
-        <v>0.4949854910373688</v>
+        <v>0.4581261873245239</v>
       </c>
       <c r="F30" t="n">
-        <v>40.23166666666668</v>
+        <v>37.54832317073172</v>
       </c>
       <c r="G30" t="n">
-        <v>4.11</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="H30" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" t="n">
         <v>0.5</v>
       </c>
-      <c r="I30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>1</v>
-      </c>
       <c r="L30" t="n">
-        <v>0.2950819672131147</v>
+        <v>0.3103448275862069</v>
       </c>
       <c r="M30" t="n">
-        <v>0.1463414634146341</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="N30" t="n">
-        <v>152.6218583583832</v>
+        <v>158.4059700965881</v>
       </c>
       <c r="O30" t="n">
-        <v>1424.9921875</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P30" t="n">
-        <v>13.2</v>
+        <v>13.5</v>
       </c>
       <c r="Q30" t="n">
         <v>20</v>
@@ -2469,10 +2469,10 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>1.466865301132202</v>
+        <v>1.224895238876343</v>
       </c>
       <c r="T30" t="n">
-        <v>151.1549906730652</v>
+        <v>157.1810719966888</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -2488,46 +2488,46 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.1086956504087902</v>
+        <v>0.1509433934069064</v>
       </c>
       <c r="D31" t="n">
-        <v>2.204506820391453e-155</v>
+        <v>2.659276018264461e-155</v>
       </c>
       <c r="E31" t="n">
-        <v>0.4693386256694794</v>
+        <v>0.5454714894294739</v>
       </c>
       <c r="F31" t="n">
-        <v>46.86125000000001</v>
+        <v>12.31171428571432</v>
       </c>
       <c r="G31" t="n">
-        <v>5.087378640776699</v>
+        <v>3.184466019417476</v>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K31" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3513513513513514</v>
       </c>
       <c r="M31" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.162303664921466</v>
       </c>
       <c r="N31" t="n">
-        <v>137.4919800758362</v>
+        <v>193.4756245613098</v>
       </c>
       <c r="O31" t="n">
-        <v>1424.99609375</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P31" t="n">
-        <v>13</v>
+        <v>13.8</v>
       </c>
       <c r="Q31" t="n">
         <v>20</v>
@@ -2536,10 +2536,10 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>1.25250244140625</v>
+        <v>1.295840978622437</v>
       </c>
       <c r="T31" t="n">
-        <v>136.239474773407</v>
+        <v>192.179780960083</v>
       </c>
       <c r="U31" t="n">
         <v>0</v>
@@ -2555,19 +2555,19 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.06399999866368003</v>
+        <v>0.073529410528763</v>
       </c>
       <c r="D32" t="n">
-        <v>1.389479870686276e-155</v>
+        <v>1.512466137089683e-155</v>
       </c>
       <c r="E32" t="n">
-        <v>0.3869301676750183</v>
+        <v>0.4342751502990723</v>
       </c>
       <c r="F32" t="n">
-        <v>54.14497505632445</v>
+        <v>42.94238991295447</v>
       </c>
       <c r="G32" t="n">
-        <v>7.36</v>
+        <v>7.81</v>
       </c>
       <c r="H32" t="n">
         <v>1</v>
@@ -2579,22 +2579,22 @@
         <v>1</v>
       </c>
       <c r="K32" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>0.3372093023255814</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="M32" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.1964285714285714</v>
       </c>
       <c r="N32" t="n">
-        <v>177.6062071323395</v>
+        <v>121.3822572231293</v>
       </c>
       <c r="O32" t="n">
-        <v>1424.99609375</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P32" t="n">
-        <v>13.3</v>
+        <v>13.5</v>
       </c>
       <c r="Q32" t="n">
         <v>20</v>
@@ -2603,10 +2603,10 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>1.489733934402466</v>
+        <v>1.264864206314087</v>
       </c>
       <c r="T32" t="n">
-        <v>176.1164700984955</v>
+        <v>120.1173901557922</v>
       </c>
       <c r="U32" t="n">
         <v>0</v>
@@ -2622,22 +2622,22 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.1958041911389311</v>
+        <v>0.251748247082987</v>
       </c>
       <c r="D33" t="n">
-        <v>3.45933709758742e-155</v>
+        <v>4.295154518309647e-155</v>
       </c>
       <c r="E33" t="n">
-        <v>0.6131397485733032</v>
+        <v>0.619636595249176</v>
       </c>
       <c r="F33" t="n">
-        <v>57.17044642857144</v>
+        <v>67.63898395721927</v>
       </c>
       <c r="G33" t="n">
-        <v>1.46814404432133</v>
+        <v>1.656509695290859</v>
       </c>
       <c r="H33" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.5</v>
       </c>
       <c r="I33" t="n">
         <v>1</v>
@@ -2646,22 +2646,22 @@
         <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>0.282051282051282</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="M33" t="n">
-        <v>0.2079207920792079</v>
+        <v>0.2253521126760563</v>
       </c>
       <c r="N33" t="n">
-        <v>164.8091218471527</v>
+        <v>195.1440138816833</v>
       </c>
       <c r="O33" t="n">
-        <v>1424.99609375</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P33" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="Q33" t="n">
         <v>20</v>
@@ -2670,10 +2670,10 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>1.475674867630005</v>
+        <v>1.455668449401855</v>
       </c>
       <c r="T33" t="n">
-        <v>163.3334443569183</v>
+        <v>193.6883425712585</v>
       </c>
       <c r="U33" t="n">
         <v>0</v>
@@ -2689,19 +2689,19 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.1686746946842794</v>
+        <v>0.2857142808721729</v>
       </c>
       <c r="D34" t="n">
-        <v>1.482225049885071e-232</v>
+        <v>1.38982761256313e-78</v>
       </c>
       <c r="E34" t="n">
-        <v>0.5662921071052551</v>
+        <v>0.6029443740844727</v>
       </c>
       <c r="F34" t="n">
-        <v>36.25755649717516</v>
+        <v>35.11720724907065</v>
       </c>
       <c r="G34" t="n">
-        <v>0.4709302325581395</v>
+        <v>1.406976744186047</v>
       </c>
       <c r="H34" t="n">
         <v>0.4</v>
@@ -2713,22 +2713,22 @@
         <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>0.2093023255813954</v>
+        <v>0.2465753424657534</v>
       </c>
       <c r="M34" t="n">
-        <v>0.1764705882352941</v>
+        <v>0.4565217391304348</v>
       </c>
       <c r="N34" t="n">
-        <v>186.9021782875061</v>
+        <v>217.3669555187225</v>
       </c>
       <c r="O34" t="n">
-        <v>1425</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P34" t="n">
-        <v>13.2</v>
+        <v>13.7</v>
       </c>
       <c r="Q34" t="n">
         <v>20</v>
@@ -2737,10 +2737,10 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>1.50193190574646</v>
+        <v>1.510351181030273</v>
       </c>
       <c r="T34" t="n">
-        <v>185.4002432823181</v>
+        <v>215.856602191925</v>
       </c>
       <c r="U34" t="n">
         <v>0</v>
@@ -2756,22 +2756,22 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.2608695603353918</v>
+        <v>0.2405063244506089</v>
       </c>
       <c r="D35" t="n">
-        <v>0.04488671857282235</v>
+        <v>0.02777353716385257</v>
       </c>
       <c r="E35" t="n">
-        <v>0.6748611927032471</v>
+        <v>0.6474072337150574</v>
       </c>
       <c r="F35" t="n">
-        <v>41.53360639972024</v>
+        <v>41.02083333333334</v>
       </c>
       <c r="G35" t="n">
-        <v>0.7495621716287215</v>
+        <v>0.6120840630472855</v>
       </c>
       <c r="H35" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I35" t="n">
         <v>1</v>
@@ -2783,19 +2783,19 @@
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>0.32</v>
+        <v>0.336734693877551</v>
       </c>
       <c r="M35" t="n">
-        <v>0.3452380952380952</v>
+        <v>0.3103448275862069</v>
       </c>
       <c r="N35" t="n">
-        <v>184.8952910900116</v>
+        <v>227.4000310897827</v>
       </c>
       <c r="O35" t="n">
-        <v>1425</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P35" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="Q35" t="n">
         <v>20</v>
@@ -2804,10 +2804,10 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>1.482797145843506</v>
+        <v>1.460640430450439</v>
       </c>
       <c r="T35" t="n">
-        <v>183.4124920368195</v>
+        <v>225.9393885135651</v>
       </c>
       <c r="U35" t="n">
         <v>0</v>
@@ -2823,19 +2823,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.2426778192678701</v>
+        <v>0.2524916895711968</v>
       </c>
       <c r="D36" t="n">
-        <v>0.06903062197415055</v>
+        <v>6.554962806708901e-79</v>
       </c>
       <c r="E36" t="n">
-        <v>0.6834411025047302</v>
+        <v>0.6158535480499268</v>
       </c>
       <c r="F36" t="n">
-        <v>17.14422705314013</v>
+        <v>34.87059288537552</v>
       </c>
       <c r="G36" t="n">
-        <v>1.206022187004754</v>
+        <v>1.787638668779715</v>
       </c>
       <c r="H36" t="n">
         <v>1</v>
@@ -2847,22 +2847,22 @@
         <v>1</v>
       </c>
       <c r="K36" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L36" t="n">
-        <v>0.34375</v>
+        <v>0.2662337662337662</v>
       </c>
       <c r="M36" t="n">
-        <v>0.3798449612403101</v>
+        <v>0.4797687861271676</v>
       </c>
       <c r="N36" t="n">
-        <v>187.1887955665588</v>
+        <v>198.508585691452</v>
       </c>
       <c r="O36" t="n">
-        <v>1425.00390625</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P36" t="n">
-        <v>13.3</v>
+        <v>13.9</v>
       </c>
       <c r="Q36" t="n">
         <v>20</v>
@@ -2871,10 +2871,10 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>1.483514785766602</v>
+        <v>1.43293571472168</v>
       </c>
       <c r="T36" t="n">
-        <v>185.7052788734436</v>
+        <v>197.075647354126</v>
       </c>
       <c r="U36" t="n">
         <v>0</v>
@@ -2890,46 +2890,46 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.2108433685121209</v>
+        <v>0.1850533758437711</v>
       </c>
       <c r="D37" t="n">
-        <v>0.02547509243889352</v>
+        <v>6.314783638207477e-79</v>
       </c>
       <c r="E37" t="n">
-        <v>0.6541558504104614</v>
+        <v>0.5938338041305542</v>
       </c>
       <c r="F37" t="n">
-        <v>44.98877137274062</v>
+        <v>38.76456043956046</v>
       </c>
       <c r="G37" t="n">
-        <v>1.219512195121951</v>
+        <v>0.7730646871686108</v>
       </c>
       <c r="H37" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="L37" t="n">
-        <v>0.261437908496732</v>
+        <v>0.25</v>
       </c>
       <c r="M37" t="n">
-        <v>0.5744680851063829</v>
+        <v>0.2156862745098039</v>
       </c>
       <c r="N37" t="n">
-        <v>238.1522080898285</v>
+        <v>159.1446752548218</v>
       </c>
       <c r="O37" t="n">
-        <v>1425.00390625</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P37" t="n">
-        <v>13.4</v>
+        <v>13.7</v>
       </c>
       <c r="Q37" t="n">
         <v>20</v>
@@ -2938,10 +2938,10 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>1.718215465545654</v>
+        <v>1.436980962753296</v>
       </c>
       <c r="T37" t="n">
-        <v>236.433990240097</v>
+        <v>157.7076916694641</v>
       </c>
       <c r="U37" t="n">
         <v>0</v>
@@ -2957,22 +2957,22 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.201058196686543</v>
+        <v>0.2229299314763278</v>
       </c>
       <c r="D38" t="n">
-        <v>9.737500401119624e-156</v>
+        <v>8.476391991707779e-79</v>
       </c>
       <c r="E38" t="n">
-        <v>0.6039879322052002</v>
+        <v>0.6034459471702576</v>
       </c>
       <c r="F38" t="n">
-        <v>15.07338235294122</v>
+        <v>31.96179054054056</v>
       </c>
       <c r="G38" t="n">
-        <v>0.5407503234152652</v>
+        <v>1.410090556274256</v>
       </c>
       <c r="H38" t="n">
-        <v>0.5</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="I38" t="n">
         <v>1</v>
@@ -2984,19 +2984,19 @@
         <v>1</v>
       </c>
       <c r="L38" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.1757575757575758</v>
       </c>
       <c r="M38" t="n">
-        <v>0.1588785046728972</v>
+        <v>0.3277310924369747</v>
       </c>
       <c r="N38" t="n">
-        <v>196.4047248363495</v>
+        <v>173.7477879524231</v>
       </c>
       <c r="O38" t="n">
-        <v>1425.0078125</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P38" t="n">
-        <v>13.3</v>
+        <v>13.6</v>
       </c>
       <c r="Q38" t="n">
         <v>20</v>
@@ -3005,10 +3005,10 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>1.5500807762146</v>
+        <v>1.440690279006958</v>
       </c>
       <c r="T38" t="n">
-        <v>194.8546423912048</v>
+        <v>172.3070952892303</v>
       </c>
       <c r="U38" t="n">
         <v>0</v>
@@ -3024,19 +3024,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.2519684990265981</v>
+        <v>0.234309618462562</v>
       </c>
       <c r="D39" t="n">
-        <v>0.04427100204850371</v>
+        <v>4.11235187953323e-155</v>
       </c>
       <c r="E39" t="n">
-        <v>0.651585578918457</v>
+        <v>0.6167111396789551</v>
       </c>
       <c r="F39" t="n">
-        <v>51.17286866201999</v>
+        <v>23.99470163703575</v>
       </c>
       <c r="G39" t="n">
-        <v>1.278761061946903</v>
+        <v>1.255162241887906</v>
       </c>
       <c r="H39" t="n">
         <v>1</v>
@@ -3045,25 +3045,25 @@
         <v>1</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v>0.3103448275862069</v>
+        <v>0.3027522935779817</v>
       </c>
       <c r="M39" t="n">
-        <v>0.3197278911564626</v>
+        <v>0.3359375</v>
       </c>
       <c r="N39" t="n">
-        <v>175.4318835735321</v>
+        <v>179.0830910205841</v>
       </c>
       <c r="O39" t="n">
-        <v>1425.01171875</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P39" t="n">
-        <v>13.2</v>
+        <v>13.8</v>
       </c>
       <c r="Q39" t="n">
         <v>20</v>
@@ -3072,10 +3072,10 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>1.479482650756836</v>
+        <v>1.216558218002319</v>
       </c>
       <c r="T39" t="n">
-        <v>173.9523987770081</v>
+        <v>177.8665306568146</v>
       </c>
       <c r="U39" t="n">
         <v>0</v>
@@ -3091,22 +3091,22 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.2260869520967865</v>
+        <v>0.2418300603596908</v>
       </c>
       <c r="D40" t="n">
-        <v>1.854559965655109e-79</v>
+        <v>1.457028417329153e-78</v>
       </c>
       <c r="E40" t="n">
-        <v>0.5178161263465881</v>
+        <v>0.6025745868682861</v>
       </c>
       <c r="F40" t="n">
-        <v>36.52914473684211</v>
+        <v>52.51057878151263</v>
       </c>
       <c r="G40" t="n">
-        <v>0.5077092511013216</v>
+        <v>1.13215859030837</v>
       </c>
       <c r="H40" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I40" t="n">
         <v>1</v>
@@ -3118,19 +3118,19 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>0.303030303030303</v>
+        <v>0.265625</v>
       </c>
       <c r="M40" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.4573643410852714</v>
       </c>
       <c r="N40" t="n">
-        <v>184.301105260849</v>
+        <v>175.5190346240997</v>
       </c>
       <c r="O40" t="n">
-        <v>1425.01171875</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P40" t="n">
-        <v>13.2</v>
+        <v>13.9</v>
       </c>
       <c r="Q40" t="n">
         <v>20</v>
@@ -3139,10 +3139,10 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>1.265569925308228</v>
+        <v>1.229546070098877</v>
       </c>
       <c r="T40" t="n">
-        <v>183.0355336666107</v>
+        <v>174.2894859313965</v>
       </c>
       <c r="U40" t="n">
         <v>0</v>
@@ -3158,22 +3158,22 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.2249240086381316</v>
+        <v>0.0507246362140307</v>
       </c>
       <c r="D41" t="n">
-        <v>5.429398294875774e-80</v>
+        <v>5.86409911537489e-163</v>
       </c>
       <c r="E41" t="n">
-        <v>0.5529953837394714</v>
+        <v>0.4579188525676727</v>
       </c>
       <c r="F41" t="n">
-        <v>46.67366854384554</v>
+        <v>39.49229885057474</v>
       </c>
       <c r="G41" t="n">
-        <v>0.3045267489711934</v>
+        <v>0.1296296296296296</v>
       </c>
       <c r="H41" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
         <v>1</v>
@@ -3185,16 +3185,16 @@
         <v>1</v>
       </c>
       <c r="L41" t="n">
-        <v>0.2950819672131147</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2424242424242424</v>
+        <v>0.1025641025641026</v>
       </c>
       <c r="N41" t="n">
-        <v>233.9566657543182</v>
+        <v>142.5459773540497</v>
       </c>
       <c r="O41" t="n">
-        <v>1425.01171875</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P41" t="n">
         <v>13.4</v>
@@ -3206,10 +3206,10 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>1.321363925933838</v>
+        <v>1.24233078956604</v>
       </c>
       <c r="T41" t="n">
-        <v>232.63529920578</v>
+        <v>141.3036441802979</v>
       </c>
       <c r="U41" t="n">
         <v>0</v>
@@ -3225,22 +3225,22 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.2288135547371446</v>
+        <v>0.2926829221072114</v>
       </c>
       <c r="D42" t="n">
-        <v>6.57725023597135e-79</v>
+        <v>0.02334892277116938</v>
       </c>
       <c r="E42" t="n">
-        <v>0.562541663646698</v>
+        <v>0.6065421104431152</v>
       </c>
       <c r="F42" t="n">
-        <v>39.94182629107985</v>
+        <v>40.86000000000001</v>
       </c>
       <c r="G42" t="n">
-        <v>0.6377142857142857</v>
+        <v>0.6697142857142857</v>
       </c>
       <c r="H42" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I42" t="n">
         <v>1</v>
@@ -3249,22 +3249,22 @@
         <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L42" t="n">
-        <v>0.2328767123287671</v>
+        <v>0.2560975609756098</v>
       </c>
       <c r="M42" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.3749999999999999</v>
       </c>
       <c r="N42" t="n">
-        <v>145.607213973999</v>
+        <v>183.410521030426</v>
       </c>
       <c r="O42" t="n">
-        <v>1425.01171875</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P42" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="Q42" t="n">
         <v>20</v>
@@ -3273,10 +3273,10 @@
         <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>1.283554077148438</v>
+        <v>1.250130891799927</v>
       </c>
       <c r="T42" t="n">
-        <v>144.323657989502</v>
+        <v>182.1603875160217</v>
       </c>
       <c r="U42" t="n">
         <v>0</v>
@@ -3292,19 +3292,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.2080536863744877</v>
+        <v>0.2363112341951184</v>
       </c>
       <c r="D43" t="n">
-        <v>4.574655955439486e-155</v>
+        <v>7.310763335123578e-79</v>
       </c>
       <c r="E43" t="n">
-        <v>0.6469773650169373</v>
+        <v>0.6416423916816711</v>
       </c>
       <c r="F43" t="n">
-        <v>44.14719696969701</v>
+        <v>38.06052650052655</v>
       </c>
       <c r="G43" t="n">
-        <v>0.7998146431881371</v>
+        <v>1.048192771084337</v>
       </c>
       <c r="H43" t="n">
         <v>1</v>
@@ -3313,25 +3313,25 @@
         <v>1</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="L43" t="n">
-        <v>0.2920353982300885</v>
+        <v>0.3103448275862069</v>
       </c>
       <c r="M43" t="n">
-        <v>0.162303664921466</v>
+        <v>0.2458100558659218</v>
       </c>
       <c r="N43" t="n">
-        <v>178.2386455535889</v>
+        <v>183.941831111908</v>
       </c>
       <c r="O43" t="n">
-        <v>1425.01953125</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P43" t="n">
-        <v>13.2</v>
+        <v>13.8</v>
       </c>
       <c r="Q43" t="n">
         <v>20</v>
@@ -3340,10 +3340,10 @@
         <v>0</v>
       </c>
       <c r="S43" t="n">
-        <v>1.479412078857422</v>
+        <v>1.238771200180054</v>
       </c>
       <c r="T43" t="n">
-        <v>176.7592308521271</v>
+        <v>182.7030580043793</v>
       </c>
       <c r="U43" t="n">
         <v>0</v>
@@ -3359,46 +3359,46 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.2246376763508192</v>
+        <v>0.2990654155646782</v>
       </c>
       <c r="D44" t="n">
-        <v>2.957452411974128e-155</v>
+        <v>0.06535170365509098</v>
       </c>
       <c r="E44" t="n">
-        <v>0.5641837120056152</v>
+        <v>0.7102271318435669</v>
       </c>
       <c r="F44" t="n">
-        <v>35.52250000000001</v>
+        <v>48.0510974443078</v>
       </c>
       <c r="G44" t="n">
-        <v>0.8105625717566016</v>
+        <v>1.013777267508611</v>
       </c>
       <c r="H44" t="n">
         <v>1</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2966101694915254</v>
       </c>
       <c r="M44" t="n">
-        <v>0.2248062015503876</v>
+        <v>0.393939393939394</v>
       </c>
       <c r="N44" t="n">
-        <v>179.8782074451447</v>
+        <v>187.4687716960907</v>
       </c>
       <c r="O44" t="n">
-        <v>1425.01953125</v>
+        <v>1444.95703125</v>
       </c>
       <c r="P44" t="n">
-        <v>13.2</v>
+        <v>13.6</v>
       </c>
       <c r="Q44" t="n">
         <v>20</v>
@@ -3407,10 +3407,10 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>1.256341695785522</v>
+        <v>1.239312648773193</v>
       </c>
       <c r="T44" t="n">
-        <v>178.6218569278717</v>
+        <v>186.2294566631317</v>
       </c>
       <c r="U44" t="n">
         <v>0</v>
@@ -3426,22 +3426,22 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.2986822803167491</v>
+        <v>0.2478386128727919</v>
       </c>
       <c r="D45" t="n">
-        <v>0.005858677697764014</v>
+        <v>0.003330175202092506</v>
       </c>
       <c r="E45" t="n">
-        <v>0.626672625541687</v>
+        <v>0.6281514167785645</v>
       </c>
       <c r="F45" t="n">
-        <v>39.44922194457067</v>
+        <v>34.03243821500308</v>
       </c>
       <c r="G45" t="n">
-        <v>0.2920208390457911</v>
+        <v>0.3035371538250617</v>
       </c>
       <c r="H45" t="n">
-        <v>0.875</v>
+        <v>0.75</v>
       </c>
       <c r="I45" t="n">
         <v>1</v>
@@ -3450,22 +3450,22 @@
         <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L45" t="n">
-        <v>0.2816901408450704</v>
+        <v>0.2368421052631579</v>
       </c>
       <c r="M45" t="n">
-        <v>0.3495934959349594</v>
+        <v>0.3220338983050848</v>
       </c>
       <c r="N45" t="n">
-        <v>196.1939218044281</v>
+        <v>201.6903517246246</v>
       </c>
       <c r="O45" t="n">
-        <v>1425.09765625</v>
+        <v>1445.1484375</v>
       </c>
       <c r="P45" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="Q45" t="n">
         <v>20</v>
@@ -3474,10 +3474,10 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>1.50542950630188</v>
+        <v>1.424128293991089</v>
       </c>
       <c r="T45" t="n">
-        <v>194.688490152359</v>
+        <v>200.2662200927734</v>
       </c>
       <c r="U45" t="n">
         <v>0</v>
@@ -3493,25 +3493,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.1705426330603209</v>
+        <v>0.2513812117613932</v>
       </c>
       <c r="D46" t="n">
-        <v>9.410118253528093e-05</v>
+        <v>0.02842566423318661</v>
       </c>
       <c r="E46" t="n">
-        <v>0.6249567866325378</v>
+        <v>0.6354157328605652</v>
       </c>
       <c r="F46" t="n">
-        <v>41.86512012012014</v>
+        <v>55.7096306818182</v>
       </c>
       <c r="G46" t="n">
-        <v>0.1855441705898643</v>
+        <v>0.3373026862364996</v>
       </c>
       <c r="H46" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="I46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
@@ -3520,19 +3520,19 @@
         <v>0.5</v>
       </c>
       <c r="L46" t="n">
-        <v>0.2298850574712644</v>
+        <v>0.2808219178082192</v>
       </c>
       <c r="M46" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.6226415094339623</v>
       </c>
       <c r="N46" t="n">
-        <v>249.3245465755463</v>
+        <v>207.9434475898743</v>
       </c>
       <c r="O46" t="n">
-        <v>1425.09765625</v>
+        <v>1445.1484375</v>
       </c>
       <c r="P46" t="n">
-        <v>13.5</v>
+        <v>13.7</v>
       </c>
       <c r="Q46" t="n">
         <v>20</v>
@@ -3541,10 +3541,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>1.473270893096924</v>
+        <v>1.241191625595093</v>
       </c>
       <c r="T46" t="n">
-        <v>247.8512737751007</v>
+        <v>206.7022526264191</v>
       </c>
       <c r="U46" t="n">
         <v>0</v>
@@ -3560,22 +3560,22 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0.2510460218202588</v>
+        <v>0.3204225307707425</v>
       </c>
       <c r="D47" t="n">
-        <v>6.516607705595573e-80</v>
+        <v>0.02074628763542984</v>
       </c>
       <c r="E47" t="n">
-        <v>0.6245467662811279</v>
+        <v>0.6796901822090149</v>
       </c>
       <c r="F47" t="n">
-        <v>42.82380952380956</v>
+        <v>32.26650825082513</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2534874451972898</v>
+        <v>0.4850538062973296</v>
       </c>
       <c r="H47" t="n">
-        <v>0.4285714285714285</v>
+        <v>1</v>
       </c>
       <c r="I47" t="n">
         <v>0</v>
@@ -3584,22 +3584,22 @@
         <v>1</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L47" t="n">
-        <v>0.3076923076923077</v>
+        <v>0.2746478873239437</v>
       </c>
       <c r="M47" t="n">
-        <v>0.2622950819672131</v>
+        <v>0.477124183006536</v>
       </c>
       <c r="N47" t="n">
-        <v>253.3274230957031</v>
+        <v>190.2458679676056</v>
       </c>
       <c r="O47" t="n">
-        <v>1425.33984375</v>
+        <v>1445.15234375</v>
       </c>
       <c r="P47" t="n">
-        <v>13.3</v>
+        <v>13.6</v>
       </c>
       <c r="Q47" t="n">
         <v>20</v>
@@ -3608,10 +3608,10 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>1.722072839736938</v>
+        <v>1.499740123748779</v>
       </c>
       <c r="T47" t="n">
-        <v>251.6053471565247</v>
+        <v>188.7461249828339</v>
       </c>
       <c r="U47" t="n">
         <v>0</v>
@@ -3627,43 +3627,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.2333333284543211</v>
+        <v>0.2236842055263159</v>
       </c>
       <c r="D48" t="n">
-        <v>1.123899409227765e-78</v>
+        <v>4.167924894556696e-155</v>
       </c>
       <c r="E48" t="n">
-        <v>0.6476296186447144</v>
+        <v>0.6185465455055237</v>
       </c>
       <c r="F48" t="n">
-        <v>32.99285714285716</v>
+        <v>46.47245121951221</v>
       </c>
       <c r="G48" t="n">
-        <v>1.381156316916488</v>
+        <v>1.019271948608137</v>
       </c>
       <c r="H48" t="n">
         <v>0.8333333333333334</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J48" t="n">
         <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L48" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="M48" t="n">
-        <v>0.1346153846153846</v>
+        <v>0.1752577319587629</v>
       </c>
       <c r="N48" t="n">
-        <v>215.6842575073242</v>
+        <v>142.4149215221405</v>
       </c>
       <c r="O48" t="n">
-        <v>1425.33984375</v>
+        <v>1445.15625</v>
       </c>
       <c r="P48" t="n">
         <v>13.5</v>
@@ -3675,10 +3675,10 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>1.462792158126831</v>
+        <v>1.243967294692993</v>
       </c>
       <c r="T48" t="n">
-        <v>214.221462726593</v>
+        <v>141.1709518432617</v>
       </c>
       <c r="U48" t="n">
         <v>0</v>
@@ -3694,46 +3694,46 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.1733333284835557</v>
+        <v>0.1874999950500001</v>
       </c>
       <c r="D49" t="n">
-        <v>5.738497806296087e-79</v>
+        <v>1.564995262624393e-155</v>
       </c>
       <c r="E49" t="n">
-        <v>0.6017470955848694</v>
+        <v>0.6401078104972839</v>
       </c>
       <c r="F49" t="n">
-        <v>24.33625000000004</v>
+        <v>37.18807692307692</v>
       </c>
       <c r="G49" t="n">
-        <v>0.7861271676300579</v>
+        <v>0.861271676300578</v>
       </c>
       <c r="H49" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="I49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J49" t="n">
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" t="n">
-        <v>0.2777777777777778</v>
+        <v>0.360655737704918</v>
       </c>
       <c r="M49" t="n">
-        <v>0.1304347826086956</v>
+        <v>0.1596638655462185</v>
       </c>
       <c r="N49" t="n">
-        <v>165.2751212120056</v>
+        <v>210.7453303337097</v>
       </c>
       <c r="O49" t="n">
-        <v>1425.33984375</v>
+        <v>1445.15625</v>
       </c>
       <c r="P49" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="Q49" t="n">
         <v>20</v>
@@ -3742,10 +3742,10 @@
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>1.48877739906311</v>
+        <v>1.231613636016846</v>
       </c>
       <c r="T49" t="n">
-        <v>163.7863421440125</v>
+        <v>209.5137135982513</v>
       </c>
       <c r="U49" t="n">
         <v>0</v>
@@ -3761,46 +3761,46 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0.2857142807663474</v>
+        <v>0.1538461512426036</v>
       </c>
       <c r="D50" t="n">
-        <v>1.10902369222975e-78</v>
+        <v>5.336379554370441e-158</v>
       </c>
       <c r="E50" t="n">
-        <v>0.649381160736084</v>
+        <v>0.5437071919441223</v>
       </c>
       <c r="F50" t="n">
-        <v>35.34602564102568</v>
+        <v>46.81274509803924</v>
       </c>
       <c r="G50" t="n">
-        <v>1.344827586206897</v>
+        <v>0.2873563218390804</v>
       </c>
       <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1</v>
+      </c>
+      <c r="L50" t="n">
         <v>0.5</v>
       </c>
-      <c r="I50" t="n">
-        <v>1</v>
-      </c>
-      <c r="J50" t="n">
-        <v>1</v>
-      </c>
-      <c r="K50" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="L50" t="n">
-        <v>0.3157894736842105</v>
-      </c>
       <c r="M50" t="n">
-        <v>0.2028985507246377</v>
+        <v>0.05797101449275362</v>
       </c>
       <c r="N50" t="n">
-        <v>172.670286655426</v>
+        <v>187.8110489845276</v>
       </c>
       <c r="O50" t="n">
-        <v>1425.33984375</v>
+        <v>1445.16015625</v>
       </c>
       <c r="P50" t="n">
-        <v>13.1</v>
+        <v>13.7</v>
       </c>
       <c r="Q50" t="n">
         <v>20</v>
@@ -3809,10 +3809,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>1.481330394744873</v>
+        <v>1.217814922332764</v>
       </c>
       <c r="T50" t="n">
-        <v>171.1889541149139</v>
+        <v>186.5932309627533</v>
       </c>
       <c r="U50" t="n">
         <v>0</v>
@@ -3828,19 +3828,19 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.29577464297684</v>
+        <v>0.3671874950076294</v>
       </c>
       <c r="D51" t="n">
-        <v>1.40176100383701e-78</v>
+        <v>0.05318774139695596</v>
       </c>
       <c r="E51" t="n">
-        <v>0.634158730506897</v>
+        <v>0.664139986038208</v>
       </c>
       <c r="F51" t="n">
-        <v>44.31494774919616</v>
+        <v>21.35137500000002</v>
       </c>
       <c r="G51" t="n">
-        <v>1.25832223701731</v>
+        <v>1.086551264980027</v>
       </c>
       <c r="H51" t="n">
         <v>1</v>
@@ -3849,25 +3849,25 @@
         <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L51" t="n">
-        <v>0.3174603174603174</v>
+        <v>0.2336448598130841</v>
       </c>
       <c r="M51" t="n">
-        <v>0.4392523364485982</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="N51" t="n">
-        <v>315.2179067134857</v>
+        <v>263.0424222946167</v>
       </c>
       <c r="O51" t="n">
-        <v>1425.6796875</v>
+        <v>1445.1640625</v>
       </c>
       <c r="P51" t="n">
-        <v>13.5</v>
+        <v>13.8</v>
       </c>
       <c r="Q51" t="n">
         <v>20</v>
@@ -3876,10 +3876,10 @@
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>1.511498689651489</v>
+        <v>1.434489727020264</v>
       </c>
       <c r="T51" t="n">
-        <v>313.7064056396484</v>
+        <v>261.6079299449921</v>
       </c>
       <c r="U51" t="n">
         <v>0</v>
@@ -3895,25 +3895,25 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.2455089778168812</v>
+        <v>0.1594202872245852</v>
       </c>
       <c r="D52" t="n">
-        <v>3.407991521845531e-79</v>
+        <v>1.335095064155259e-157</v>
       </c>
       <c r="E52" t="n">
-        <v>0.6236441135406494</v>
+        <v>0.5645071864128113</v>
       </c>
       <c r="F52" t="n">
-        <v>52.71924735111438</v>
+        <v>39.86342857142861</v>
       </c>
       <c r="G52" t="n">
-        <v>0.4314720812182741</v>
+        <v>0.2059463379260334</v>
       </c>
       <c r="H52" t="n">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -3922,19 +3922,19 @@
         <v>1</v>
       </c>
       <c r="L52" t="n">
-        <v>0.2682926829268293</v>
+        <v>0.2058823529411765</v>
       </c>
       <c r="M52" t="n">
-        <v>0.2173913043478261</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="N52" t="n">
-        <v>176.9254086017609</v>
+        <v>203.0529260635376</v>
       </c>
       <c r="O52" t="n">
-        <v>1425.6796875</v>
+        <v>1445.171875</v>
       </c>
       <c r="P52" t="n">
-        <v>13.2</v>
+        <v>13.8</v>
       </c>
       <c r="Q52" t="n">
         <v>20</v>
@@ -3943,10 +3943,10 @@
         <v>0</v>
       </c>
       <c r="S52" t="n">
-        <v>1.504750967025757</v>
+        <v>1.292034864425659</v>
       </c>
       <c r="T52" t="n">
-        <v>175.4206552505493</v>
+        <v>201.7608885765076</v>
       </c>
       <c r="U52" t="n">
         <v>0</v>
@@ -3962,46 +3962,46 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.3603603558433772</v>
+        <v>0.3749999953233688</v>
       </c>
       <c r="D53" t="n">
-        <v>0.04679951705481336</v>
+        <v>0.03338087509600714</v>
       </c>
       <c r="E53" t="n">
-        <v>0.6791532039642334</v>
+        <v>0.6651744842529297</v>
       </c>
       <c r="F53" t="n">
-        <v>39.58948446528373</v>
+        <v>35.30533967391307</v>
       </c>
       <c r="G53" t="n">
-        <v>0.5096051227321238</v>
+        <v>0.6013874066168623</v>
       </c>
       <c r="H53" t="n">
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="I53" t="n">
         <v>1</v>
       </c>
       <c r="J53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K53" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>0.3089430894308943</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="M53" t="n">
-        <v>0.452054794520548</v>
+        <v>0.388888888888889</v>
       </c>
       <c r="N53" t="n">
-        <v>233.0190327167511</v>
+        <v>225.9946026802063</v>
       </c>
       <c r="O53" t="n">
-        <v>1425.6796875</v>
+        <v>1445.40234375</v>
       </c>
       <c r="P53" t="n">
-        <v>13.4</v>
+        <v>13.7</v>
       </c>
       <c r="Q53" t="n">
         <v>20</v>
@@ -4010,10 +4010,10 @@
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>1.48765230178833</v>
+        <v>1.44616436958313</v>
       </c>
       <c r="T53" t="n">
-        <v>231.5313785076141</v>
+        <v>224.5484359264374</v>
       </c>
       <c r="U53" t="n">
         <v>0</v>
@@ -4029,46 +4029,46 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.2910052860558215</v>
+        <v>0.3428571380349388</v>
       </c>
       <c r="D54" t="n">
-        <v>0.06899407273030436</v>
+        <v>0.08414974269172384</v>
       </c>
       <c r="E54" t="n">
-        <v>0.6660365462303162</v>
+        <v>0.6761053204536438</v>
       </c>
       <c r="F54" t="n">
-        <v>37.73903483309147</v>
+        <v>43.7644774590164</v>
       </c>
       <c r="G54" t="n">
-        <v>0.8366445916114791</v>
+        <v>0.6769683590875644</v>
       </c>
       <c r="H54" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="I54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="L54" t="n">
-        <v>0.2147651006711409</v>
+        <v>0.2822580645161291</v>
       </c>
       <c r="M54" t="n">
-        <v>0.4244604316546763</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="N54" t="n">
-        <v>203.4117324352264</v>
+        <v>264.5489459037781</v>
       </c>
       <c r="O54" t="n">
-        <v>1425.6796875</v>
+        <v>1445.41015625</v>
       </c>
       <c r="P54" t="n">
-        <v>13.4</v>
+        <v>13.9</v>
       </c>
       <c r="Q54" t="n">
         <v>20</v>
@@ -4077,10 +4077,10 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>1.287887334823608</v>
+        <v>1.1799476146698</v>
       </c>
       <c r="T54" t="n">
-        <v>202.123842716217</v>
+        <v>263.3689961433411</v>
       </c>
       <c r="U54" t="n">
         <v>0</v>
@@ -4096,25 +4096,25 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0.2322946131130176</v>
+        <v>0.04528301686009265</v>
       </c>
       <c r="D55" t="n">
-        <v>0.01058202302624076</v>
+        <v>3.396921629371405e-239</v>
       </c>
       <c r="E55" t="n">
-        <v>0.6578117609024048</v>
+        <v>0.5777973532676697</v>
       </c>
       <c r="F55" t="n">
-        <v>23.14378947368425</v>
+        <v>-67.21749999999997</v>
       </c>
       <c r="G55" t="n">
-        <v>0.4870633893919793</v>
+        <v>0.1966364812419146</v>
       </c>
       <c r="H55" t="n">
-        <v>0.3157894736842105</v>
+        <v>1</v>
       </c>
       <c r="I55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J55" t="n">
         <v>1</v>
@@ -4123,19 +4123,19 @@
         <v>1</v>
       </c>
       <c r="L55" t="n">
-        <v>0.2403846153846154</v>
+        <v>0.2352941176470588</v>
       </c>
       <c r="M55" t="n">
-        <v>0.2391304347826087</v>
+        <v>0.05660377358490565</v>
       </c>
       <c r="N55" t="n">
-        <v>198.3057036399841</v>
+        <v>206.7777540683746</v>
       </c>
       <c r="O55" t="n">
-        <v>1425.6796875</v>
+        <v>1445.4140625</v>
       </c>
       <c r="P55" t="n">
-        <v>13.4</v>
+        <v>13.7</v>
       </c>
       <c r="Q55" t="n">
         <v>20</v>
@@ -4144,10 +4144,10 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>1.253013610839844</v>
+        <v>1.216771125793457</v>
       </c>
       <c r="T55" t="n">
-        <v>197.0526881217957</v>
+        <v>205.5609812736511</v>
       </c>
       <c r="U55" t="n">
         <v>0</v>
@@ -4163,46 +4163,46 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0.09420289672757828</v>
+        <v>0.2239999955205689</v>
       </c>
       <c r="D56" t="n">
-        <v>1.595125071640276e-239</v>
+        <v>1.850791334670095e-79</v>
       </c>
       <c r="E56" t="n">
-        <v>0.5541946887969971</v>
+        <v>0.6431059837341309</v>
       </c>
       <c r="F56" t="n">
-        <v>31.10813725490198</v>
+        <v>29.25229508196725</v>
       </c>
       <c r="G56" t="n">
-        <v>0.1544352265475431</v>
+        <v>0.4767070835992342</v>
       </c>
       <c r="H56" t="n">
-        <v>0.1904761904761905</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="I56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J56" t="n">
         <v>1</v>
       </c>
       <c r="K56" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L56" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="M56" t="n">
-        <v>0.1139240506329114</v>
+        <v>0.2481203007518797</v>
       </c>
       <c r="N56" t="n">
-        <v>197.0316779613495</v>
+        <v>202.7357501983643</v>
       </c>
       <c r="O56" t="n">
-        <v>1425.6796875</v>
+        <v>1445.41796875</v>
       </c>
       <c r="P56" t="n">
-        <v>13.4</v>
+        <v>13.6</v>
       </c>
       <c r="Q56" t="n">
         <v>20</v>
@@ -4211,10 +4211,10 @@
         <v>0</v>
       </c>
       <c r="S56" t="n">
-        <v>1.232639789581299</v>
+        <v>1.25344705581665</v>
       </c>
       <c r="T56" t="n">
-        <v>195.7990362644196</v>
+        <v>201.4823005199432</v>
       </c>
       <c r="U56" t="n">
         <v>0</v>
@@ -4230,19 +4230,19 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>0.2675367008268378</v>
+        <v>0.2618657898993093</v>
       </c>
       <c r="D57" t="n">
-        <v>0.01055434144634028</v>
+        <v>0.005945899370026579</v>
       </c>
       <c r="E57" t="n">
-        <v>0.6141224503517151</v>
+        <v>0.6275182962417603</v>
       </c>
       <c r="F57" t="n">
-        <v>51.36713793103448</v>
+        <v>42.95492300049679</v>
       </c>
       <c r="G57" t="n">
-        <v>0.3552722260509993</v>
+        <v>0.3242591316333563</v>
       </c>
       <c r="H57" t="n">
         <v>0.3333333333333333</v>
@@ -4254,22 +4254,22 @@
         <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L57" t="n">
-        <v>0.2361111111111111</v>
+        <v>0.2</v>
       </c>
       <c r="M57" t="n">
-        <v>0.2063492063492063</v>
+        <v>0.2</v>
       </c>
       <c r="N57" t="n">
-        <v>297.6989760398865</v>
+        <v>224.5429842472076</v>
       </c>
       <c r="O57" t="n">
-        <v>1425.8203125</v>
+        <v>1445.953125</v>
       </c>
       <c r="P57" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="Q57" t="n">
         <v>20</v>
@@ -4278,10 +4278,10 @@
         <v>0</v>
       </c>
       <c r="S57" t="n">
-        <v>1.279675245285034</v>
+        <v>1.222887277603149</v>
       </c>
       <c r="T57" t="n">
-        <v>296.4192986488342</v>
+        <v>223.3200941085815</v>
       </c>
       <c r="U57" t="n">
         <v>0</v>
@@ -4297,46 +4297,46 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0.1517857102427456</v>
+        <v>0.2380952331039188</v>
       </c>
       <c r="D58" t="n">
-        <v>1.117533984565559e-79</v>
+        <v>9.320458944274172e-79</v>
       </c>
       <c r="E58" t="n">
-        <v>0.5478999018669128</v>
+        <v>0.6378589272499084</v>
       </c>
       <c r="F58" t="n">
-        <v>17.29523255813953</v>
+        <v>26.06043860713419</v>
       </c>
       <c r="G58" t="n">
-        <v>0.4362850971922246</v>
+        <v>1.163066954643629</v>
       </c>
       <c r="H58" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
       </c>
       <c r="K58" t="n">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="L58" t="n">
-        <v>0.25</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="M58" t="n">
-        <v>0.1935483870967742</v>
+        <v>0.4623655913978494</v>
       </c>
       <c r="N58" t="n">
-        <v>211.3234415054321</v>
+        <v>194.4991102218628</v>
       </c>
       <c r="O58" t="n">
-        <v>1425.8203125</v>
+        <v>1445.95703125</v>
       </c>
       <c r="P58" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="Q58" t="n">
         <v>20</v>
@@ -4345,10 +4345,10 @@
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>1.227201223373413</v>
+        <v>1.244938611984253</v>
       </c>
       <c r="T58" t="n">
-        <v>210.0962376594543</v>
+        <v>193.2541687488556</v>
       </c>
       <c r="U58" t="n">
         <v>0</v>
@@ -4364,46 +4364,46 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.2134831420275218</v>
+        <v>0.2535211218091649</v>
       </c>
       <c r="D59" t="n">
-        <v>1.151793102877015e-79</v>
+        <v>0.02103885804841746</v>
       </c>
       <c r="E59" t="n">
-        <v>0.5395029187202454</v>
+        <v>0.5801204442977905</v>
       </c>
       <c r="F59" t="n">
-        <v>-1.349080459770079</v>
+        <v>29.81879310344829</v>
       </c>
       <c r="G59" t="n">
-        <v>0.4393939393939394</v>
+        <v>1.21969696969697</v>
       </c>
       <c r="H59" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="I59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J59" t="n">
         <v>1</v>
       </c>
       <c r="K59" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L59" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.2781954887218045</v>
       </c>
       <c r="M59" t="n">
-        <v>0.1129032258064516</v>
+        <v>0.3043478260869565</v>
       </c>
       <c r="N59" t="n">
-        <v>173.9121851921082</v>
+        <v>193.0151836872101</v>
       </c>
       <c r="O59" t="n">
-        <v>1425.8203125</v>
+        <v>1445.9609375</v>
       </c>
       <c r="P59" t="n">
-        <v>13.1</v>
+        <v>13.6</v>
       </c>
       <c r="Q59" t="n">
         <v>20</v>
@@ -4412,10 +4412,10 @@
         <v>0</v>
       </c>
       <c r="S59" t="n">
-        <v>1.502098083496094</v>
+        <v>1.442703723907471</v>
       </c>
       <c r="T59" t="n">
-        <v>172.4100849628448</v>
+        <v>191.5724775791168</v>
       </c>
       <c r="U59" t="n">
         <v>0</v>
@@ -4431,46 +4431,46 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0.2780410700483417</v>
+        <v>0.275752769192161</v>
       </c>
       <c r="D60" t="n">
-        <v>0.01450794484019664</v>
+        <v>0.03097275134609704</v>
       </c>
       <c r="E60" t="n">
-        <v>0.6303671598434448</v>
+        <v>0.6212339401245117</v>
       </c>
       <c r="F60" t="n">
-        <v>35.22313725490199</v>
+        <v>31.86911612599906</v>
       </c>
       <c r="G60" t="n">
-        <v>0.4454926624737945</v>
+        <v>0.5310971348707197</v>
       </c>
       <c r="H60" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I60" t="n">
         <v>1</v>
       </c>
       <c r="J60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K60" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L60" t="n">
-        <v>0.245398773006135</v>
+        <v>0.2298136645962733</v>
       </c>
       <c r="M60" t="n">
-        <v>0.458128078817734</v>
+        <v>0.6716417910447761</v>
       </c>
       <c r="N60" t="n">
-        <v>188.1288003921509</v>
+        <v>342.0660843849182</v>
       </c>
       <c r="O60" t="n">
-        <v>1425.8203125</v>
+        <v>1446.21484375</v>
       </c>
       <c r="P60" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="Q60" t="n">
         <v>20</v>
@@ -4479,10 +4479,10 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>1.221950531005859</v>
+        <v>1.211202144622803</v>
       </c>
       <c r="T60" t="n">
-        <v>186.9068479537964</v>
+        <v>340.8548800945282</v>
       </c>
       <c r="U60" t="n">
         <v>0</v>
@@ -4498,46 +4498,46 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0.1363636329350322</v>
+        <v>0.1212121183147843</v>
       </c>
       <c r="D61" t="n">
-        <v>2.775544290086747e-155</v>
+        <v>5.434222959060843e-79</v>
       </c>
       <c r="E61" t="n">
-        <v>0.5160923004150391</v>
+        <v>0.4991749823093414</v>
       </c>
       <c r="F61" t="n">
-        <v>22.2842391304348</v>
+        <v>54.79465184049081</v>
       </c>
       <c r="G61" t="n">
-        <v>2.506072874493927</v>
+        <v>3.396761133603239</v>
       </c>
       <c r="H61" t="n">
         <v>1</v>
       </c>
       <c r="I61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J61" t="n">
         <v>1</v>
       </c>
       <c r="K61" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L61" t="n">
-        <v>0.313953488372093</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="M61" t="n">
-        <v>0.1772151898734177</v>
+        <v>0.3233082706766917</v>
       </c>
       <c r="N61" t="n">
-        <v>185.7766962051392</v>
+        <v>196.8808014392853</v>
       </c>
       <c r="O61" t="n">
-        <v>1425.8203125</v>
+        <v>1446.21484375</v>
       </c>
       <c r="P61" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="Q61" t="n">
         <v>20</v>
@@ -4546,10 +4546,10 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>1.277440547943115</v>
+        <v>1.255117177963257</v>
       </c>
       <c r="T61" t="n">
-        <v>184.4992532730103</v>
+        <v>195.6256816387177</v>
       </c>
       <c r="U61" t="n">
         <v>0</v>
@@ -4565,25 +4565,25 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0.2068965470585613</v>
+        <v>0.1526717507907466</v>
       </c>
       <c r="D62" t="n">
-        <v>1.525420446765144e-155</v>
+        <v>2.041150620072487e-155</v>
       </c>
       <c r="E62" t="n">
-        <v>0.4929231405258179</v>
+        <v>0.6374655365943909</v>
       </c>
       <c r="F62" t="n">
-        <v>49.72587264150945</v>
+        <v>36.98561538461541</v>
       </c>
       <c r="G62" t="n">
-        <v>0.6525</v>
+        <v>0.9225</v>
       </c>
       <c r="H62" t="n">
         <v>1</v>
       </c>
       <c r="I62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J62" t="n">
         <v>1</v>
@@ -4592,19 +4592,19 @@
         <v>1</v>
       </c>
       <c r="L62" t="n">
-        <v>0.2285714285714286</v>
+        <v>0.3877551020408163</v>
       </c>
       <c r="M62" t="n">
-        <v>0.1</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="N62" t="n">
-        <v>217.5486812591553</v>
+        <v>157.4113132953644</v>
       </c>
       <c r="O62" t="n">
-        <v>1425.8203125</v>
+        <v>1446.21484375</v>
       </c>
       <c r="P62" t="n">
-        <v>13.6</v>
+        <v>13.5</v>
       </c>
       <c r="Q62" t="n">
         <v>20</v>
@@ -4613,10 +4613,10 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>1.420284271240234</v>
+        <v>1.350200176239014</v>
       </c>
       <c r="T62" t="n">
-        <v>216.1283946037292</v>
+        <v>156.061110496521</v>
       </c>
       <c r="U62" t="n">
         <v>0</v>
@@ -4632,46 +4632,46 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0.2279792703267203</v>
+        <v>0.1752577276474653</v>
       </c>
       <c r="D63" t="n">
-        <v>2.698386591461445e-79</v>
+        <v>4.999600024564736e-156</v>
       </c>
       <c r="E63" t="n">
-        <v>0.5203997492790222</v>
+        <v>0.5119909644126892</v>
       </c>
       <c r="F63" t="n">
-        <v>49.29145833333337</v>
+        <v>47.07205399061036</v>
       </c>
       <c r="G63" t="n">
-        <v>0.5202231520223152</v>
+        <v>0.4909344490934449</v>
       </c>
       <c r="H63" t="n">
         <v>0.25</v>
       </c>
       <c r="I63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J63" t="n">
         <v>1</v>
       </c>
       <c r="K63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L63" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3125</v>
       </c>
       <c r="M63" t="n">
-        <v>0.1150442477876106</v>
+        <v>0.08256880733944955</v>
       </c>
       <c r="N63" t="n">
-        <v>145.0687770843506</v>
+        <v>177.8854670524597</v>
       </c>
       <c r="O63" t="n">
-        <v>1425.8203125</v>
+        <v>1446.21484375</v>
       </c>
       <c r="P63" t="n">
-        <v>13.2</v>
+        <v>13.8</v>
       </c>
       <c r="Q63" t="n">
         <v>20</v>
@@ -4680,10 +4680,10 @@
         <v>0</v>
       </c>
       <c r="S63" t="n">
-        <v>1.456096887588501</v>
+        <v>1.214670181274414</v>
       </c>
       <c r="T63" t="n">
-        <v>143.6126778125763</v>
+        <v>176.6707942485809</v>
       </c>
       <c r="U63" t="n">
         <v>0</v>
@@ -4699,19 +4699,19 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0.3092783456052716</v>
+        <v>0.2583025782029112</v>
       </c>
       <c r="D64" t="n">
-        <v>3.551652806380462e-155</v>
+        <v>0.02514370313572025</v>
       </c>
       <c r="E64" t="n">
-        <v>0.6491305232048035</v>
+        <v>0.6672975420951843</v>
       </c>
       <c r="F64" t="n">
-        <v>50.49725000000004</v>
+        <v>39.89187180796733</v>
       </c>
       <c r="G64" t="n">
-        <v>0.8819672131147541</v>
+        <v>1.567213114754098</v>
       </c>
       <c r="H64" t="n">
         <v>0.75</v>
@@ -4723,22 +4723,22 @@
         <v>1</v>
       </c>
       <c r="K64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L64" t="n">
-        <v>0.3582089552238806</v>
+        <v>0.336</v>
       </c>
       <c r="M64" t="n">
-        <v>0.1911764705882353</v>
+        <v>0.2537313432835821</v>
       </c>
       <c r="N64" t="n">
-        <v>187.9322338104248</v>
+        <v>209.5704565048218</v>
       </c>
       <c r="O64" t="n">
-        <v>1425.8203125</v>
+        <v>1446.21484375</v>
       </c>
       <c r="P64" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="Q64" t="n">
         <v>20</v>
@@ -4747,10 +4747,10 @@
         <v>0</v>
       </c>
       <c r="S64" t="n">
-        <v>1.500192642211914</v>
+        <v>1.221551418304443</v>
       </c>
       <c r="T64" t="n">
-        <v>186.4320387840271</v>
+        <v>208.3489022254944</v>
       </c>
       <c r="U64" t="n">
         <v>0</v>
@@ -4766,19 +4766,19 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0.259999995018</v>
+        <v>0.2743362783271988</v>
       </c>
       <c r="D65" t="n">
-        <v>1.005424523454277e-78</v>
+        <v>0.0414682325579625</v>
       </c>
       <c r="E65" t="n">
-        <v>0.592657208442688</v>
+        <v>0.6343826055526733</v>
       </c>
       <c r="F65" t="n">
-        <v>53.62308327825514</v>
+        <v>53.11579184100421</v>
       </c>
       <c r="G65" t="n">
-        <v>1.280561122244489</v>
+        <v>1.547094188376753</v>
       </c>
       <c r="H65" t="n">
         <v>1</v>
@@ -4790,22 +4790,22 @@
         <v>1</v>
       </c>
       <c r="K65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L65" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.35</v>
       </c>
       <c r="M65" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2156862745098039</v>
       </c>
       <c r="N65" t="n">
-        <v>168.4373672008514</v>
+        <v>155.6822469234467</v>
       </c>
       <c r="O65" t="n">
-        <v>1425.8203125</v>
+        <v>1446.21484375</v>
       </c>
       <c r="P65" t="n">
-        <v>13.3</v>
+        <v>13.5</v>
       </c>
       <c r="Q65" t="n">
         <v>20</v>
@@ -4814,10 +4814,10 @@
         <v>0</v>
       </c>
       <c r="S65" t="n">
-        <v>1.283151865005493</v>
+        <v>1.248746871948242</v>
       </c>
       <c r="T65" t="n">
-        <v>167.1542131900787</v>
+        <v>154.4334971904755</v>
       </c>
       <c r="U65" t="n">
         <v>0</v>
@@ -4833,19 +4833,19 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0.2292490070021404</v>
+        <v>0.3294117598351404</v>
       </c>
       <c r="D66" t="n">
-        <v>0.02219715813919129</v>
+        <v>0.03913077173831421</v>
       </c>
       <c r="E66" t="n">
-        <v>0.5993309020996094</v>
+        <v>0.6727531552314758</v>
       </c>
       <c r="F66" t="n">
-        <v>34.30561919504646</v>
+        <v>56.7633287292818</v>
       </c>
       <c r="G66" t="n">
-        <v>0.8682559598494354</v>
+        <v>0.7641154328732748</v>
       </c>
       <c r="H66" t="n">
         <v>0.6666666666666666</v>
@@ -4857,22 +4857,22 @@
         <v>0</v>
       </c>
       <c r="K66" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="L66" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="M66" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="N66" t="n">
-        <v>152.0732223987579</v>
+        <v>161.0369536876678</v>
       </c>
       <c r="O66" t="n">
-        <v>1425.8203125</v>
+        <v>1446.21484375</v>
       </c>
       <c r="P66" t="n">
-        <v>13.1</v>
+        <v>13.6</v>
       </c>
       <c r="Q66" t="n">
         <v>20</v>
@@ -4881,10 +4881,10 @@
         <v>0</v>
       </c>
       <c r="S66" t="n">
-        <v>1.220553874969482</v>
+        <v>1.218591690063477</v>
       </c>
       <c r="T66" t="n">
-        <v>150.8526666164398</v>
+        <v>159.8183596134186</v>
       </c>
       <c r="U66" t="n">
         <v>0</v>
@@ -4900,46 +4900,46 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0.2317596517010813</v>
+        <v>0.2809917305539239</v>
       </c>
       <c r="D67" t="n">
-        <v>1.243482204168198e-78</v>
+        <v>0.03998047557520408</v>
       </c>
       <c r="E67" t="n">
-        <v>0.6747742891311646</v>
+        <v>0.6766796112060547</v>
       </c>
       <c r="F67" t="n">
-        <v>50.6308424908425</v>
+        <v>37.66029411764708</v>
       </c>
       <c r="G67" t="n">
-        <v>0.8178082191780822</v>
+        <v>0.8945205479452055</v>
       </c>
       <c r="H67" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L67" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="M67" t="n">
-        <v>0.101123595505618</v>
+        <v>0.2366412213740458</v>
       </c>
       <c r="N67" t="n">
-        <v>1057.302765607834</v>
+        <v>178.8530859947205</v>
       </c>
       <c r="O67" t="n">
-        <v>1427.69921875</v>
+        <v>1446.21484375</v>
       </c>
       <c r="P67" t="n">
-        <v>11.6</v>
+        <v>13.5</v>
       </c>
       <c r="Q67" t="n">
         <v>20</v>
@@ -4948,10 +4948,10 @@
         <v>0</v>
       </c>
       <c r="S67" t="n">
-        <v>1.523171663284302</v>
+        <v>1.55723237991333</v>
       </c>
       <c r="T67" t="n">
-        <v>1055.779591560364</v>
+        <v>177.2958514690399</v>
       </c>
       <c r="U67" t="n">
         <v>0</v>
@@ -4967,46 +4967,46 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.1161290305098855</v>
+        <v>0.2051282020216963</v>
       </c>
       <c r="D68" t="n">
-        <v>4.762308121761521e-79</v>
+        <v>9.656944879633529e-79</v>
       </c>
       <c r="E68" t="n">
-        <v>0.4599381983280182</v>
+        <v>0.5352259278297424</v>
       </c>
       <c r="F68" t="n">
-        <v>7.826848635235763</v>
+        <v>13.3386363636364</v>
       </c>
       <c r="G68" t="n">
-        <v>7.007874015748031</v>
+        <v>3.204724409448819</v>
       </c>
       <c r="H68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
       </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L68" t="n">
-        <v>0.272</v>
+        <v>0.3559322033898305</v>
       </c>
       <c r="M68" t="n">
-        <v>0.3617021276595745</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="N68" t="n">
-        <v>173.943398475647</v>
+        <v>209.3800349235535</v>
       </c>
       <c r="O68" t="n">
-        <v>1427.69921875</v>
+        <v>1446.21484375</v>
       </c>
       <c r="P68" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="Q68" t="n">
         <v>20</v>
@@ -5015,10 +5015,10 @@
         <v>0</v>
       </c>
       <c r="S68" t="n">
-        <v>1.281460285186768</v>
+        <v>1.227649927139282</v>
       </c>
       <c r="T68" t="n">
-        <v>172.661936044693</v>
+        <v>208.152382850647</v>
       </c>
       <c r="U68" t="n">
         <v>0</v>

</xml_diff>